<commit_message>
Add live uniform listing for 72114 from fresh ledger export
00_Uniform_Listing_72114.xlsx: full 72114 Uniforms account from the
9-Jun TechOne export, 103 lines, $26,236.42 ex-GST, 22 service codes,
one row per line with the four-limb criteria columns.

  L1 Svc/PK validated against svc_map: 98 GREEN (PK matches service
    home), 5 AMBER (off-home or unmapped).
  L3 Evidence from attachment flag: 57 of 103 lines carry no attachment
    (RED), 46 have attachments (pending sighting).
  L2 NA seeded: IPWEA -$10,650.27 (GJ078546) flagged to 73542
    Professional Membership, the rest uniforms in 72114.

Summary sheet carries the RAG rollup and attachment coverage. Listing
TOTAL recalc-verified at $26,236.42. Register 72114 row points to the
listing; reviewed-$ stays the $1,059.76 Reali subset. Source export
preserved in New/ as raw intake. Bundle manifest regenerated and
strict-verified.

https://claude.ai/code/session_01DsAVs3nwb32qeSApHrKLXa
</commit_message>
<xml_diff>
--- a/00_Account_Review_Register.xlsx
+++ b/00_Account_Review_Register.xlsx
@@ -202,13 +202,13 @@
     <t xml:space="preserve">N/A</t>
   </si>
   <si>
-    <t xml:space="preserve">3-Jun Reali PK split $1,059.76 confirmed subset (~4%). GJ SOURCE NOW SIGHTED (Document Reconstruction, doc 202603161072172000000001, ledger 26SLACT): a BALANCED multi-account recode batch (nets $0.00). Its 72114 block credits $10,650.27 from 1-20001-72114 narrated 'Institute of Public Works Engineering Au' (IPWEA) and DEBITS the same $10,650.27 across 16 service-level 72114 (Uniforms) PKs. CONCERN: if the $10,650.27 is a genuine IPWEA professional charge it should leave 72114 entirely (73542 Professional Membership most likely, or 73541 Conferences / 73544 Training), not be redistributed WITHIN Uniforms. Wider Reali standing-order set ($17,288.98) now provided (C00223414 zip), not yet worked.</t>
+    <t xml:space="preserve">3-Jun Reali PK split $1,059.76 confirmed subset (~4%). GJ SOURCE NOW SIGHTED (Document Reconstruction, doc 202603161072172000000001, ledger 26SLACT): a BALANCED multi-account recode batch (nets $0.00). Its 72114 block credits $10,650.27 from 1-20001-72114 narrated 'Institute of Public Works Engineering Au' (IPWEA) and DEBITS the same $10,650.27 across 16 service-level 72114 (Uniforms) PKs. CONCERN: if the $10,650.27 is a genuine IPWEA professional charge it should leave 72114 entirely (73542 Professional Membership most likely, or 73541 Conferences / 73544 Training), not be redistributed WITHIN Uniforms. Wider Reali standing-order set ($17,288.98) now provided (C00223414 zip), not yet worked. LIVE LISTING 9-Jun: 00_Uniform_Listing_72114.xlsx built from fresh TechOne export - full account 103 lines $26,236.42, 22 service codes. L1 Svc/PK 98 GREEN / 5 AMBER (off-home/unmapped); 57 of 103 lines have NO attachment (RED evidence); 46 have attachments (pending sighting). IPWEA -$10,650.27 (GJ078546) flagged to 73542. Reviewed-$ in this register stays the $1,059.76 Reali subset; the listing is the live per-line state.</t>
   </si>
   <si>
     <t xml:space="preserve">1 Confirm whether the reconstruction batch is POSTED or PROPOSED; if posted, the IPWEA $10,650.27 is already spread across Uniforms service PKs. 2 Obtain the underlying IPWEA invoice to confirm nature (membership vs conference vs training) and set destination (73542/73541/73544); it should not sit in 72114. 3 Work the now-provided Reali set at full scope. 4 Confirm net-movement vs full-reversal format. Same batch also shows other apparent miscodes outside scope (e.g. Empire Office Furniture $4,300 in 73544 Training).</t>
   </si>
   <si>
-    <t xml:space="preserve">NA72114_Scope_Note.md; Document_Reconstruction (GJ source) sighted; C00223414 Reali set provided</t>
+    <t xml:space="preserve">NA72114_Scope_Note.md; Document_Reconstruction (GJ source) sighted; C00223414 Reali set provided; 00_Uniform_Listing_72114.xlsx (full account, per-line)</t>
   </si>
   <si>
     <t xml:space="preserve">73140</t>

</xml_diff>

<commit_message>
73211 evidence pass 2: file 15 Barbs/Wallum/RST small-series invoices supplied
Correction: the C00273057 and C00278314 intakes were first mis-triaged as
out-of-scope landscape docs; on re-match against the ledger every invoice is a
73211 small-series line. 15 sighted exact to GL on the x1.1 test (+$11,458.60):
11 Barbs Trees (00031079-00031269), 3 Wallum (00059183/00059890/00060386),
RST 00001394. ABN checksums PASS (Barbs 89 859 104 277, Wallum 92 086 722 456,
RST 21 627 796 435). No GST errors.

Filed canonically with SHA-256; the 00031079/085/086 GAP row closed; manifest
small-series GAP restated to the 6 unsighted lines ($3,133.70) + Provac $2,050.
Verification-record addendum 2, EvidencePass log, and register row updated.
Bundle manifest regenerated, strict verify PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E2DraJoXMLMxk1NyzJ13Vc
</commit_message>
<xml_diff>
--- a/00_Account_Review_Register.xlsx
+++ b/00_Account_Review_Register.xlsx
@@ -1821,7 +1821,7 @@
       </c>
       <c r="L21" s="19" t="inlineStr">
         <is>
-          <t>Residual evidence GAP (~$5,505 quantified + EWN): small series 00059013/00031055/79/85/86/00060617/47 ($2,438.20), Provac INV-00037183 ($2,050), Telstra Dec-25 ($727.95), EWN INV-14768 (amount tbc); Ausecology $450 residual + vendor ABN. SCOPE: fresh 17-Jun export totals $267,532.19 vs register $236,378.27, delta $31,153.92 (suspected added P11/P12 lines incl 8 Org Risk Consulting WHS invoices INV-250714/811-813/910-913 present in intake but absent from 73211 ledger refs) - reconcile before changing scope. F1-F7 and candidate rulings still Spero's. | 18-Jun: NEW GAPs - 00001190 cemeteries standing order $500 (P12, PK000083, doc 1240297) and Destination Trails INV-0356 $24,340 (P12, above $20k floor, feeds F2). Small-series remainder now 00031079/85/86 + 00060647 ($1,313.80). Telstra Dec-25 already closed via Document Reconstruction 97; vendor PDF C00255407 now in _Sources_18-Jun-2026/ can upgrade it to a vendor sighting later.</t>
+          <t>Residual evidence GAP (~$5,505 quantified + EWN): small series 00059013/00031055/79/85/86/00060617/47 ($2,438.20), Provac INV-00037183 ($2,050), Telstra Dec-25 ($727.95), EWN INV-14768 (amount tbc); Ausecology $450 residual + vendor ABN. SCOPE: fresh 17-Jun export totals $267,532.19 vs register $236,378.27, delta $31,153.92 (suspected added P11/P12 lines incl 8 Org Risk Consulting WHS invoices INV-250714/811-813/910-913 present in intake but absent from 73211 ledger refs) - reconcile before changing scope. F1-F7 and candidate rulings still Spero's. | 18-Jun: NEW GAPs - 00001190 cemeteries standing order $500 (P12, PK000083, doc 1240297) and Destination Trails INV-0356 $24,340 (P12, above $20k floor, feeds F2). Small-series remainder now 00031079/85/86 + 00060647 ($1,313.80). Telstra Dec-25 already closed via Document Reconstruction 97; vendor PDF C00255407 now in _Sources_18-Jun-2026/ can upgrade it to a vendor sighting later. | 18-Jun pass 2: 15 Barbs/Wallum/RST small-series invoices SIGHTED exact (+$11,458.60), ABNs PASS; residual small-series 6 lines $3,133.70 (00059199/568/569, 00060647/756, 00061080) + Provac $2,050.</t>
         </is>
       </c>
       <c r="M21" s="19" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="O21" s="19" t="inlineStr">
         <is>
-          <t>18-Jun-2026 (evidence pass)</t>
+          <t>18-Jun-2026 (evidence pass 2)</t>
         </is>
       </c>
     </row>

</xml_diff>